<commit_message>
Section audit: up to five reviewers per section
Five name and email slots per section with a signed-up count; open slots
highlighted; Summary lists every reviewer. Columns are found by name so the
formulas follow the layout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqfFtE1Qb9uN7QDcn19AvE
</commit_message>
<xml_diff>
--- a/docs/HCM_Academy_Section_Audit.xlsx
+++ b/docs/HCM_Academy_Section_Audit.xlsx
@@ -600,7 +600,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Sign up. On the Sign-up tab, put your name and email in Reviewer 1 or Reviewer 2 for a section that still has an open slot (highlighted). Two reviewers per section, at most.</t>
+          <t>Sign up. On the Sign-up tab, put your name and email in the next open Reviewer slot (highlighted) for a section. Up to five reviewers per section; split the course topics between you and put your name in the Reviewer column of each row you audit.</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="B2" s="6">
-        <f>TRIM('Sign-up'!E2&amp;IF(LEN('Sign-up'!G2)&gt;0,", "&amp;'Sign-up'!G2,""))</f>
+        <f>MID(IF(LEN('Sign-up'!E2)&gt;0,", "&amp;'Sign-up'!E2,"")&amp;IF(LEN('Sign-up'!G2)&gt;0,", "&amp;'Sign-up'!G2,"")&amp;IF(LEN('Sign-up'!I2)&gt;0,", "&amp;'Sign-up'!I2,"")&amp;IF(LEN('Sign-up'!K2)&gt;0,", "&amp;'Sign-up'!K2,"")&amp;IF(LEN('Sign-up'!M2)&gt;0,", "&amp;'Sign-up'!M2,""),3,500)</f>
         <v/>
       </c>
       <c r="C2" s="6" t="n">
@@ -1273,7 +1273,7 @@
         <v/>
       </c>
       <c r="K2" s="6">
-        <f>'Sign-up'!J2</f>
+        <f>'Sign-up'!Q2</f>
         <v/>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="B3" s="6">
-        <f>TRIM('Sign-up'!E3&amp;IF(LEN('Sign-up'!G3)&gt;0,", "&amp;'Sign-up'!G3,""))</f>
+        <f>MID(IF(LEN('Sign-up'!E3)&gt;0,", "&amp;'Sign-up'!E3,"")&amp;IF(LEN('Sign-up'!G3)&gt;0,", "&amp;'Sign-up'!G3,"")&amp;IF(LEN('Sign-up'!I3)&gt;0,", "&amp;'Sign-up'!I3,"")&amp;IF(LEN('Sign-up'!K3)&gt;0,", "&amp;'Sign-up'!K3,"")&amp;IF(LEN('Sign-up'!M3)&gt;0,", "&amp;'Sign-up'!M3,""),3,500)</f>
         <v/>
       </c>
       <c r="C3" s="6" t="n">
@@ -1319,7 +1319,7 @@
         <v/>
       </c>
       <c r="K3" s="6">
-        <f>'Sign-up'!J3</f>
+        <f>'Sign-up'!Q3</f>
         <v/>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>TRIM('Sign-up'!E4&amp;IF(LEN('Sign-up'!G4)&gt;0,", "&amp;'Sign-up'!G4,""))</f>
+        <f>MID(IF(LEN('Sign-up'!E4)&gt;0,", "&amp;'Sign-up'!E4,"")&amp;IF(LEN('Sign-up'!G4)&gt;0,", "&amp;'Sign-up'!G4,"")&amp;IF(LEN('Sign-up'!I4)&gt;0,", "&amp;'Sign-up'!I4,"")&amp;IF(LEN('Sign-up'!K4)&gt;0,", "&amp;'Sign-up'!K4,"")&amp;IF(LEN('Sign-up'!M4)&gt;0,", "&amp;'Sign-up'!M4,""),3,500)</f>
         <v/>
       </c>
       <c r="C4" s="6" t="n">
@@ -1365,7 +1365,7 @@
         <v/>
       </c>
       <c r="K4" s="6">
-        <f>'Sign-up'!J4</f>
+        <f>'Sign-up'!Q4</f>
         <v/>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>TRIM('Sign-up'!E5&amp;IF(LEN('Sign-up'!G5)&gt;0,", "&amp;'Sign-up'!G5,""))</f>
+        <f>MID(IF(LEN('Sign-up'!E5)&gt;0,", "&amp;'Sign-up'!E5,"")&amp;IF(LEN('Sign-up'!G5)&gt;0,", "&amp;'Sign-up'!G5,"")&amp;IF(LEN('Sign-up'!I5)&gt;0,", "&amp;'Sign-up'!I5,"")&amp;IF(LEN('Sign-up'!K5)&gt;0,", "&amp;'Sign-up'!K5,"")&amp;IF(LEN('Sign-up'!M5)&gt;0,", "&amp;'Sign-up'!M5,""),3,500)</f>
         <v/>
       </c>
       <c r="C5" s="6" t="n">
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="K5" s="6">
-        <f>'Sign-up'!J5</f>
+        <f>'Sign-up'!Q5</f>
         <v/>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>TRIM('Sign-up'!E6&amp;IF(LEN('Sign-up'!G6)&gt;0,", "&amp;'Sign-up'!G6,""))</f>
+        <f>MID(IF(LEN('Sign-up'!E6)&gt;0,", "&amp;'Sign-up'!E6,"")&amp;IF(LEN('Sign-up'!G6)&gt;0,", "&amp;'Sign-up'!G6,"")&amp;IF(LEN('Sign-up'!I6)&gt;0,", "&amp;'Sign-up'!I6,"")&amp;IF(LEN('Sign-up'!K6)&gt;0,", "&amp;'Sign-up'!K6,"")&amp;IF(LEN('Sign-up'!M6)&gt;0,", "&amp;'Sign-up'!M6,""),3,500)</f>
         <v/>
       </c>
       <c r="C6" s="6" t="n">
@@ -1457,7 +1457,7 @@
         <v/>
       </c>
       <c r="K6" s="6">
-        <f>'Sign-up'!J6</f>
+        <f>'Sign-up'!Q6</f>
         <v/>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>TRIM('Sign-up'!E7&amp;IF(LEN('Sign-up'!G7)&gt;0,", "&amp;'Sign-up'!G7,""))</f>
+        <f>MID(IF(LEN('Sign-up'!E7)&gt;0,", "&amp;'Sign-up'!E7,"")&amp;IF(LEN('Sign-up'!G7)&gt;0,", "&amp;'Sign-up'!G7,"")&amp;IF(LEN('Sign-up'!I7)&gt;0,", "&amp;'Sign-up'!I7,"")&amp;IF(LEN('Sign-up'!K7)&gt;0,", "&amp;'Sign-up'!K7,"")&amp;IF(LEN('Sign-up'!M7)&gt;0,", "&amp;'Sign-up'!M7,""),3,500)</f>
         <v/>
       </c>
       <c r="C7" s="6" t="n">
@@ -1503,7 +1503,7 @@
         <v/>
       </c>
       <c r="K7" s="6">
-        <f>'Sign-up'!J7</f>
+        <f>'Sign-up'!Q7</f>
         <v/>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>TRIM('Sign-up'!E8&amp;IF(LEN('Sign-up'!G8)&gt;0,", "&amp;'Sign-up'!G8,""))</f>
+        <f>MID(IF(LEN('Sign-up'!E8)&gt;0,", "&amp;'Sign-up'!E8,"")&amp;IF(LEN('Sign-up'!G8)&gt;0,", "&amp;'Sign-up'!G8,"")&amp;IF(LEN('Sign-up'!I8)&gt;0,", "&amp;'Sign-up'!I8,"")&amp;IF(LEN('Sign-up'!K8)&gt;0,", "&amp;'Sign-up'!K8,"")&amp;IF(LEN('Sign-up'!M8)&gt;0,", "&amp;'Sign-up'!M8,""),3,500)</f>
         <v/>
       </c>
       <c r="C8" s="6" t="n">
@@ -1549,7 +1549,7 @@
         <v/>
       </c>
       <c r="K8" s="6">
-        <f>'Sign-up'!J8</f>
+        <f>'Sign-up'!Q8</f>
         <v/>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="B9" s="6">
-        <f>TRIM('Sign-up'!E9&amp;IF(LEN('Sign-up'!G9)&gt;0,", "&amp;'Sign-up'!G9,""))</f>
+        <f>MID(IF(LEN('Sign-up'!E9)&gt;0,", "&amp;'Sign-up'!E9,"")&amp;IF(LEN('Sign-up'!G9)&gt;0,", "&amp;'Sign-up'!G9,"")&amp;IF(LEN('Sign-up'!I9)&gt;0,", "&amp;'Sign-up'!I9,"")&amp;IF(LEN('Sign-up'!K9)&gt;0,", "&amp;'Sign-up'!K9,"")&amp;IF(LEN('Sign-up'!M9)&gt;0,", "&amp;'Sign-up'!M9,""),3,500)</f>
         <v/>
       </c>
       <c r="C9" s="6" t="n">
@@ -1595,7 +1595,7 @@
         <v/>
       </c>
       <c r="K9" s="6">
-        <f>'Sign-up'!J9</f>
+        <f>'Sign-up'!Q9</f>
         <v/>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1812,12 +1812,19 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1863,30 +1870,65 @@
       </c>
       <c r="I1" s="5" t="inlineStr">
         <is>
+          <t>Reviewer 3</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Reviewer 3 email</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Reviewer 4</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Reviewer 4 email</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Reviewer 5</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Reviewer 5 email</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>Reviewers signed up</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
           <t>Target date</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>Audit status</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="R1" s="5" t="inlineStr">
         <is>
           <t>Audited so far</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="S1" s="5" t="inlineStr">
         <is>
           <t>Section verdict</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="T1" s="5" t="inlineStr">
         <is>
           <t>Section notes</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="U1" s="5" t="inlineStr">
         <is>
           <t>Go to section</t>
         </is>
@@ -1915,19 +1957,29 @@
       <c r="F2" s="7" t="inlineStr"/>
       <c r="G2" s="7" t="inlineStr"/>
       <c r="H2" s="7" t="inlineStr"/>
-      <c r="I2" s="8" t="inlineStr"/>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K2" s="9">
-        <f>IFERROR(COUNTA('00 Start Here'!J2:J10)/9,0)</f>
-        <v/>
-      </c>
+      <c r="I2" s="7" t="inlineStr"/>
+      <c r="J2" s="7" t="inlineStr"/>
+      <c r="K2" s="7" t="inlineStr"/>
       <c r="L2" s="7" t="inlineStr"/>
       <c r="M2" s="7" t="inlineStr"/>
-      <c r="N2" s="10" t="inlineStr">
+      <c r="N2" s="7" t="inlineStr"/>
+      <c r="O2" s="6">
+        <f>(LEN(E2)&gt;0)+(LEN(G2)&gt;0)+(LEN(I2)&gt;0)+(LEN(K2)&gt;0)+(LEN(M2)&gt;0)&amp;" of 5"</f>
+        <v/>
+      </c>
+      <c r="P2" s="8" t="inlineStr"/>
+      <c r="Q2" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="R2" s="9">
+        <f>IFERROR(COUNTA('00 Start Here'!J2:J10)/9,0)</f>
+        <v/>
+      </c>
+      <c r="S2" s="7" t="inlineStr"/>
+      <c r="T2" s="7" t="inlineStr"/>
+      <c r="U2" s="10" t="inlineStr">
         <is>
           <t>Open tab</t>
         </is>
@@ -1956,19 +2008,29 @@
       <c r="F3" s="7" t="inlineStr"/>
       <c r="G3" s="7" t="inlineStr"/>
       <c r="H3" s="7" t="inlineStr"/>
-      <c r="I3" s="8" t="inlineStr"/>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K3" s="9">
-        <f>IFERROR(COUNTA('01 Hiring'!J2:J20)/19,0)</f>
-        <v/>
-      </c>
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr"/>
+      <c r="K3" s="7" t="inlineStr"/>
       <c r="L3" s="7" t="inlineStr"/>
       <c r="M3" s="7" t="inlineStr"/>
-      <c r="N3" s="10" t="inlineStr">
+      <c r="N3" s="7" t="inlineStr"/>
+      <c r="O3" s="6">
+        <f>(LEN(E3)&gt;0)+(LEN(G3)&gt;0)+(LEN(I3)&gt;0)+(LEN(K3)&gt;0)+(LEN(M3)&gt;0)&amp;" of 5"</f>
+        <v/>
+      </c>
+      <c r="P3" s="8" t="inlineStr"/>
+      <c r="Q3" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="R3" s="9">
+        <f>IFERROR(COUNTA('01 Hiring'!J2:J20)/19,0)</f>
+        <v/>
+      </c>
+      <c r="S3" s="7" t="inlineStr"/>
+      <c r="T3" s="7" t="inlineStr"/>
+      <c r="U3" s="10" t="inlineStr">
         <is>
           <t>Open tab</t>
         </is>
@@ -1997,19 +2059,29 @@
       <c r="F4" s="7" t="inlineStr"/>
       <c r="G4" s="7" t="inlineStr"/>
       <c r="H4" s="7" t="inlineStr"/>
-      <c r="I4" s="8" t="inlineStr"/>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K4" s="9">
-        <f>IFERROR(COUNTA('02 Payroll'!J2:J13)/12,0)</f>
-        <v/>
-      </c>
+      <c r="I4" s="7" t="inlineStr"/>
+      <c r="J4" s="7" t="inlineStr"/>
+      <c r="K4" s="7" t="inlineStr"/>
       <c r="L4" s="7" t="inlineStr"/>
       <c r="M4" s="7" t="inlineStr"/>
-      <c r="N4" s="10" t="inlineStr">
+      <c r="N4" s="7" t="inlineStr"/>
+      <c r="O4" s="6">
+        <f>(LEN(E4)&gt;0)+(LEN(G4)&gt;0)+(LEN(I4)&gt;0)+(LEN(K4)&gt;0)+(LEN(M4)&gt;0)&amp;" of 5"</f>
+        <v/>
+      </c>
+      <c r="P4" s="8" t="inlineStr"/>
+      <c r="Q4" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="R4" s="9">
+        <f>IFERROR(COUNTA('02 Payroll'!J2:J13)/12,0)</f>
+        <v/>
+      </c>
+      <c r="S4" s="7" t="inlineStr"/>
+      <c r="T4" s="7" t="inlineStr"/>
+      <c r="U4" s="10" t="inlineStr">
         <is>
           <t>Open tab</t>
         </is>
@@ -2038,19 +2110,29 @@
       <c r="F5" s="7" t="inlineStr"/>
       <c r="G5" s="7" t="inlineStr"/>
       <c r="H5" s="7" t="inlineStr"/>
-      <c r="I5" s="8" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K5" s="9">
-        <f>IFERROR(COUNTA('03 Assignments'!J2:J14)/13,0)</f>
-        <v/>
-      </c>
+      <c r="I5" s="7" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr"/>
+      <c r="K5" s="7" t="inlineStr"/>
       <c r="L5" s="7" t="inlineStr"/>
       <c r="M5" s="7" t="inlineStr"/>
-      <c r="N5" s="10" t="inlineStr">
+      <c r="N5" s="7" t="inlineStr"/>
+      <c r="O5" s="6">
+        <f>(LEN(E5)&gt;0)+(LEN(G5)&gt;0)+(LEN(I5)&gt;0)+(LEN(K5)&gt;0)+(LEN(M5)&gt;0)&amp;" of 5"</f>
+        <v/>
+      </c>
+      <c r="P5" s="8" t="inlineStr"/>
+      <c r="Q5" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="R5" s="9">
+        <f>IFERROR(COUNTA('03 Assignments'!J2:J14)/13,0)</f>
+        <v/>
+      </c>
+      <c r="S5" s="7" t="inlineStr"/>
+      <c r="T5" s="7" t="inlineStr"/>
+      <c r="U5" s="10" t="inlineStr">
         <is>
           <t>Open tab</t>
         </is>
@@ -2079,19 +2161,29 @@
       <c r="F6" s="7" t="inlineStr"/>
       <c r="G6" s="7" t="inlineStr"/>
       <c r="H6" s="7" t="inlineStr"/>
-      <c r="I6" s="8" t="inlineStr"/>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K6" s="9">
-        <f>IFERROR(COUNTA('04 Leave'!J2:J6)/5,0)</f>
-        <v/>
-      </c>
+      <c r="I6" s="7" t="inlineStr"/>
+      <c r="J6" s="7" t="inlineStr"/>
+      <c r="K6" s="7" t="inlineStr"/>
       <c r="L6" s="7" t="inlineStr"/>
       <c r="M6" s="7" t="inlineStr"/>
-      <c r="N6" s="10" t="inlineStr">
+      <c r="N6" s="7" t="inlineStr"/>
+      <c r="O6" s="6">
+        <f>(LEN(E6)&gt;0)+(LEN(G6)&gt;0)+(LEN(I6)&gt;0)+(LEN(K6)&gt;0)+(LEN(M6)&gt;0)&amp;" of 5"</f>
+        <v/>
+      </c>
+      <c r="P6" s="8" t="inlineStr"/>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="R6" s="9">
+        <f>IFERROR(COUNTA('04 Leave'!J2:J6)/5,0)</f>
+        <v/>
+      </c>
+      <c r="S6" s="7" t="inlineStr"/>
+      <c r="T6" s="7" t="inlineStr"/>
+      <c r="U6" s="10" t="inlineStr">
         <is>
           <t>Open tab</t>
         </is>
@@ -2120,19 +2212,29 @@
       <c r="F7" s="7" t="inlineStr"/>
       <c r="G7" s="7" t="inlineStr"/>
       <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="8" t="inlineStr"/>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K7" s="9">
-        <f>IFERROR(COUNTA('05 Costing'!J2:J6)/5,0)</f>
-        <v/>
-      </c>
+      <c r="I7" s="7" t="inlineStr"/>
+      <c r="J7" s="7" t="inlineStr"/>
+      <c r="K7" s="7" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr"/>
       <c r="M7" s="7" t="inlineStr"/>
-      <c r="N7" s="10" t="inlineStr">
+      <c r="N7" s="7" t="inlineStr"/>
+      <c r="O7" s="6">
+        <f>(LEN(E7)&gt;0)+(LEN(G7)&gt;0)+(LEN(I7)&gt;0)+(LEN(K7)&gt;0)+(LEN(M7)&gt;0)&amp;" of 5"</f>
+        <v/>
+      </c>
+      <c r="P7" s="8" t="inlineStr"/>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="R7" s="9">
+        <f>IFERROR(COUNTA('05 Costing'!J2:J6)/5,0)</f>
+        <v/>
+      </c>
+      <c r="S7" s="7" t="inlineStr"/>
+      <c r="T7" s="7" t="inlineStr"/>
+      <c r="U7" s="10" t="inlineStr">
         <is>
           <t>Open tab</t>
         </is>
@@ -2161,19 +2263,29 @@
       <c r="F8" s="7" t="inlineStr"/>
       <c r="G8" s="7" t="inlineStr"/>
       <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="8" t="inlineStr"/>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K8" s="9">
-        <f>IFERROR(COUNTA('06 Students and Faculty'!J2:J12)/11,0)</f>
-        <v/>
-      </c>
+      <c r="I8" s="7" t="inlineStr"/>
+      <c r="J8" s="7" t="inlineStr"/>
+      <c r="K8" s="7" t="inlineStr"/>
       <c r="L8" s="7" t="inlineStr"/>
       <c r="M8" s="7" t="inlineStr"/>
-      <c r="N8" s="10" t="inlineStr">
+      <c r="N8" s="7" t="inlineStr"/>
+      <c r="O8" s="6">
+        <f>(LEN(E8)&gt;0)+(LEN(G8)&gt;0)+(LEN(I8)&gt;0)+(LEN(K8)&gt;0)+(LEN(M8)&gt;0)&amp;" of 5"</f>
+        <v/>
+      </c>
+      <c r="P8" s="8" t="inlineStr"/>
+      <c r="Q8" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="R8" s="9">
+        <f>IFERROR(COUNTA('06 Students and Faculty'!J2:J12)/11,0)</f>
+        <v/>
+      </c>
+      <c r="S8" s="7" t="inlineStr"/>
+      <c r="T8" s="7" t="inlineStr"/>
+      <c r="U8" s="10" t="inlineStr">
         <is>
           <t>Open tab</t>
         </is>
@@ -2202,26 +2314,36 @@
       <c r="F9" s="7" t="inlineStr"/>
       <c r="G9" s="7" t="inlineStr"/>
       <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="8" t="inlineStr"/>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K9" s="9">
-        <f>IFERROR(COUNTA('07 Records'!J2:J6)/5,0)</f>
-        <v/>
-      </c>
+      <c r="I9" s="7" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr"/>
+      <c r="K9" s="7" t="inlineStr"/>
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr"/>
-      <c r="N9" s="10" t="inlineStr">
+      <c r="N9" s="7" t="inlineStr"/>
+      <c r="O9" s="6">
+        <f>(LEN(E9)&gt;0)+(LEN(G9)&gt;0)+(LEN(I9)&gt;0)+(LEN(K9)&gt;0)+(LEN(M9)&gt;0)&amp;" of 5"</f>
+        <v/>
+      </c>
+      <c r="P9" s="8" t="inlineStr"/>
+      <c r="Q9" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="R9" s="9">
+        <f>IFERROR(COUNTA('07 Records'!J2:J6)/5,0)</f>
+        <v/>
+      </c>
+      <c r="S9" s="7" t="inlineStr"/>
+      <c r="T9" s="7" t="inlineStr"/>
+      <c r="U9" s="10" t="inlineStr">
         <is>
           <t>Open tab</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J2:J9">
+  <conditionalFormatting sqref="Q2:Q9">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
@@ -2231,23 +2353,43 @@
       <formula>LEN(E2)=0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G9">
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>LEN(G2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I9">
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>LEN(I2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:K9">
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>LEN(K2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M2:M9">
+    <cfRule type="expression" priority="6" dxfId="1">
+      <formula>LEN(M2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="J2:J9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." type="list">
+    <dataValidation sqref="Q2:Q9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." type="list">
       <formula1>=Lists!$E$1:$E$3</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." type="list">
+    <dataValidation sqref="S2:S9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." type="list">
       <formula1>=Lists!$F$1:$F$6</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>